<commit_message>
Complete pending system test cases
</commit_message>
<xml_diff>
--- a/output/testing/uthai-smash-system-test-cases.xlsx
+++ b/output/testing/uthai-smash-system-test-cases.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปผล" sheetId="1" r:id="R9caf2c2d4f2e47b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R1bcabd649df84b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปผล" sheetId="1" r:id="R8c32cee560b24b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R7dbec9f1a21d49b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -388,7 +388,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +399,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DE"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +410,7 @@
         <x:color rgb="FF946200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
@@ -721,7 +721,7 @@
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:f>COUNTIF('Test Cases'!$I$6:$I$50,"PASS")</x:f>
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C6" s="13" t="n">
         <x:f>COUNTIF('Test Cases'!$I$6:$I$50,"FAIL")</x:f>
@@ -729,7 +729,7 @@
       </x:c>
       <x:c r="D6" s="13" t="n">
         <x:f>COUNTIF('Test Cases'!$I$6:$I$50,"NOT RUN")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="52"/>
       <x:c r="F6" s="17" t="str">
@@ -832,10 +832,10 @@
       </x:c>
       <x:c r="F12" s="52"/>
       <x:c r="G12" s="30" t="str">
-        <x:v>TC-016 · FAIL</x:v>
+        <x:v>TC-034 · FAIL</x:v>
       </x:c>
       <x:c r="H12" s="29" t="str">
-        <x:v>บอร์ดคิวใช้ชื่อย่อซ้ำจนแยกคนไม่ได้ ควรแสดงชื่อเต็ม</x:v>
+        <x:v>ระบบบันทึกเพียงสถานะส่งหลักฐาน ไม่มีไฟล์จริงให้ Admin เปิดตรวจ</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
@@ -860,10 +860,10 @@
       </x:c>
       <x:c r="F13" s="52"/>
       <x:c r="G13" s="30" t="str">
-        <x:v>TC-017 · FAIL</x:v>
+        <x:v>TC-043 · FAIL</x:v>
       </x:c>
       <x:c r="H13" s="29" t="str">
-        <x:v>จำนวน Client ในข้อความ WebSocket ค้าง แม้ LIVE badge เปลี่ยน</x:v>
+        <x:v>บอร์ด 20 คิวบน 1366×768 ต้องเลื่อนลง แม้ Full HD แสดงครบ</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
@@ -887,12 +887,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="52"/>
-      <x:c r="G14" s="30" t="str">
-        <x:v>TC-034 · NOT RUN</x:v>
-      </x:c>
-      <x:c r="H14" s="29" t="str">
-        <x:v>ยังไม่ได้อัปโหลดไฟล์หลักฐานจริง</x:v>
-      </x:c>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="29"/>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
       <x:c r="A15" s="23" t="str">
@@ -915,12 +911,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="52"/>
-      <x:c r="G15" s="30" t="str">
-        <x:v>TC-043 · NOT RUN</x:v>
-      </x:c>
-      <x:c r="H15" s="29" t="str">
-        <x:v>ยังไม่ได้ทำ Visual regression ที่ 10/20 คิวและหลายขนาดจอ</x:v>
-      </x:c>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="29"/>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
       <x:c r="A16" s="23" t="str">
@@ -943,12 +935,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="52"/>
-      <x:c r="G16" s="30" t="str">
-        <x:v>TC-044 · NOT RUN</x:v>
-      </x:c>
-      <x:c r="H16" s="29" t="str">
-        <x:v>ยังไม่ได้ตรวจไฟล์รูปทวงเงินที่ดาวน์โหลด</x:v>
-      </x:c>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="29"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="23" t="str">
@@ -1022,7 +1010,7 @@
       </x:c>
       <x:c r="F19" s="52"/>
       <x:c r="G19" s="46" t="str">
-        <x:v>Core flow ใช้งานได้ครบตั้งแต่สมาชิก → เช็คอิน → คิว/สนาม → เบิกลูก/ซื้อของ → สรุปและรับชำระ พร้อมการบันทึก JSON และ Real-time ควรแก้ชื่อเต็มบน Board ก่อนเปิดใช้งานจริง และเพิ่ม automated browser tests สำหรับไฟล์ดาวน์โหลด/อัปโหลดกับหน้าจอคิวหนาแน่น</x:v>
+        <x:v>Core flow ผ่านครบและเคสค้างถูกทดสอบแล้ว 3 รายการ รูปทวงเงินใช้งานได้ทั้งแบบรวมและรายคน จุดที่ต้องแก้ก่อนใช้งานจริงคือเก็บไฟล์หลักฐานจริงให้ Admin เปิดดู และปรับบอร์ด 20 คิวให้พอดีกับจอ 1366×768</x:v>
       </x:c>
       <x:c r="H19" s="47"/>
     </x:row>
@@ -1036,11 +1024,11 @@
       </x:c>
       <x:c r="C20" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A20,'Test Cases'!$I$6:$I$50,C$12)</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D20" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A20,'Test Cases'!$I$6:$I$50,D$12)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A20,'Test Cases'!$I$6:$I$50,E$12)</x:f>
@@ -1132,15 +1120,15 @@
       </x:c>
       <x:c r="C24" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A24,'Test Cases'!$I$6:$I$50,C$12)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D24" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A24,'Test Cases'!$I$6:$I$50,D$12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E24" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A24,'Test Cases'!$I$6:$I$50,E$12)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="52"/>
       <x:c r="G24" s="52"/>
@@ -1256,11 +1244,11 @@
       </x:c>
       <x:c r="D29" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A29,'Test Cases'!$I$6:$I$50,D$12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E29" s="24" t="n">
         <x:f>COUNTIFS('Test Cases'!$B$6:$B$50,A29,'Test Cases'!$I$6:$I$50,E$12)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="52"/>
       <x:c r="G29" s="52"/>
@@ -1972,16 +1960,16 @@
         <x:v>เห็นชื่อเต็มของผู้เล่นทั้ง 4 คน</x:v>
       </x:c>
       <x:c r="H21" s="61" t="str">
-        <x:v>แสดงเพียง ทดสอบ · ทดสอบ · ทดสอบ · ทดสอบ</x:v>
+        <x:v>แก้แล้วและทดสอบซ้ำ Board แสดงชื่อเต็มของผู้เล่นทั้ง 4 คน</x:v>
       </x:c>
       <x:c r="I21" s="62" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="J21" s="62" t="str">
-        <x:v>พบจาก Board UI</x:v>
+        <x:v>UI retest · commit 40a37dc</x:v>
       </x:c>
       <x:c r="K21" s="62" t="str">
-        <x:v>20 ต.ค. 2569</x:v>
+        <x:v>21 ต.ค. 2569</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="66" customHeight="1">
@@ -2007,16 +1995,16 @@
         <x:v>จำนวน Client ตรงกันทุกตำแหน่ง</x:v>
       </x:c>
       <x:c r="H22" s="61" t="str">
-        <x:v>Header แสดงหลาย Client แต่ข้อความในเนื้อหายังค้างที่ 0</x:v>
+        <x:v>แก้แล้ว จำนวนจอใน Board เปลี่ยน 1 → 2 และกลับเป็น 1 ตรงกับ LIVE badge</x:v>
       </x:c>
       <x:c r="I22" s="62" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="J22" s="62" t="str">
-        <x:v>พบจาก Board UI</x:v>
+        <x:v>UI + automated retest</x:v>
       </x:c>
       <x:c r="K22" s="62" t="str">
-        <x:v>20 ต.ค. 2569</x:v>
+        <x:v>21 ต.ค. 2569</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="66" customHeight="1">
@@ -2602,16 +2590,16 @@
         <x:v>Admin เห็นหลักฐานที่ส่ง</x:v>
       </x:c>
       <x:c r="H39" s="61" t="str">
-        <x:v>ยังไม่ได้ทดสอบการอัปโหลดไฟล์จริง</x:v>
+        <x:v>เลือกไฟล์และส่งได้ แต่ Backend เก็บเพียง submittedAt ไม่มีไฟล์หรือ URL ให้ Admin เปิดดู</x:v>
       </x:c>
       <x:c r="I39" s="62" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="J39" s="62" t="str">
-        <x:v>ต้องใช้ไฟล์ทดสอบเฉพาะ</x:v>
+        <x:v>UI upload + GET /api/state</x:v>
       </x:c>
       <x:c r="K39" s="62" t="str">
-        <x:v>-</x:v>
+        <x:v>21 ต.ค. 2569</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="66" customHeight="1">
@@ -2917,16 +2905,16 @@
         <x:v>ไม่ล้นจอและยังอ่านชื่อได้</x:v>
       </x:c>
       <x:c r="H48" s="61" t="str">
-        <x:v>ยังไม่ได้รันทดสอบข้อมูลหนาแน่นและทุก breakpoint</x:v>
+        <x:v>10 คิวพอดีที่ 1920×1080 และ 1366×768; 20 คิวพอดีเฉพาะ 1920×1080 แต่ 1366×768 สูง 931px จึงต้องเลื่อน</x:v>
       </x:c>
       <x:c r="I48" s="62" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="J48" s="62" t="str">
-        <x:v>ควรเพิ่ม visual regression</x:v>
+        <x:v>Responsive UI · 4 combinations</x:v>
       </x:c>
       <x:c r="K48" s="62" t="str">
-        <x:v>-</x:v>
+        <x:v>21 ต.ค. 2569</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="66" customHeight="1">
@@ -2952,16 +2940,16 @@
         <x:v>ได้ไฟล์รูปที่อ่านง่ายและยอดถูกต้อง</x:v>
       </x:c>
       <x:c r="H49" s="61" t="str">
-        <x:v>ยังไม่ได้ทดสอบไฟล์ดาวน์โหลดจริง</x:v>
+        <x:v>ดาวน์โหลดภาพรวมและรายคนสำเร็จ PNG 1080×1080; ยอดรวม ฿95 และรายคน ฿23.75 ถูกต้อง</x:v>
       </x:c>
       <x:c r="I49" s="62" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="J49" s="62" t="str">
-        <x:v>ต้องตรวจไฟล์ภาพปลายทาง</x:v>
+        <x:v>Browser download + visual check</x:v>
       </x:c>
       <x:c r="K49" s="62" t="str">
-        <x:v>-</x:v>
+        <x:v>21 ต.ค. 2569</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="66" customHeight="1">
@@ -3011,7 +2999,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ab0d978d49f496e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcd6b8487c7d4a24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>